<commit_message>
feat: Services, Packages, Addon, and Refunds. feat: New service added for application to load on the localdb for local ordering. feat: New Packages for application to get and save on localdb to allow customers to order packages. feat: Addons are added for the application to pull addons (WIP) no actual data so validation/verification is needed. feat: Added Addon repository to allow the refunds UI Sheet to call and refund a sale. fix: Fixed refund sheet to be able to call the addon repository. feat: Added new Addon controller to separate the sheet from the dashboard controller.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\TEMP\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73C14D01-72FF-4821-8EFB-D628684ECCCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CC08D1-D961-4D79-B55C-DE3D0097FE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="142">
   <si>
     <t>API Integration &amp; Testing Checklist</t>
   </si>
@@ -431,6 +431,21 @@
   </si>
   <si>
     <t>Used to show the amount collected by the cashier inside the receipt.</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Used to get services for the application to be able to use.</t>
+  </si>
+  <si>
+    <t>Used to get the active Addons in the server to use on the application (This causes errors on the server when adding there so double check is needed to properly show the data on the application).</t>
+  </si>
+  <si>
+    <t>Used to get the packages from the server to use onto the application.</t>
+  </si>
+  <si>
+    <t>Used to refund the orders. The user is required to manually input the OR number as well as the reason for the refund.</t>
   </si>
 </sst>
 </file>
@@ -512,14 +527,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -882,14 +897,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -927,7 +942,7 @@
       <c r="E4" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="4" t="s">
         <v>119</v>
       </c>
     </row>
@@ -947,7 +962,7 @@
       <c r="E5" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="4" t="s">
         <v>120</v>
       </c>
     </row>
@@ -967,7 +982,7 @@
       <c r="E6" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="4" t="s">
         <v>121</v>
       </c>
     </row>
@@ -987,7 +1002,7 @@
       <c r="E7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="6"/>
+      <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -1005,7 +1020,7 @@
       <c r="E8" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" s="4" t="s">
         <v>122</v>
       </c>
     </row>
@@ -1025,7 +1040,7 @@
       <c r="E9" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="6"/>
+      <c r="F9" s="4"/>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -1043,7 +1058,7 @@
       <c r="E10" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" s="4" t="s">
         <v>123</v>
       </c>
     </row>
@@ -1063,7 +1078,7 @@
       <c r="E11" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" s="4" t="s">
         <v>124</v>
       </c>
     </row>
@@ -1083,7 +1098,7 @@
       <c r="E12" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="4" t="s">
         <v>125</v>
       </c>
     </row>
@@ -1103,7 +1118,7 @@
       <c r="E13" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" s="4" t="s">
         <v>126</v>
       </c>
     </row>
@@ -1123,7 +1138,7 @@
       <c r="E14" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" s="4" t="s">
         <v>127</v>
       </c>
     </row>
@@ -1143,7 +1158,7 @@
       <c r="E15" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" s="4" t="s">
         <v>128</v>
       </c>
     </row>
@@ -1163,7 +1178,7 @@
       <c r="E16" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" s="4" t="s">
         <v>129</v>
       </c>
     </row>
@@ -1183,7 +1198,7 @@
       <c r="E17" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
@@ -1201,7 +1216,7 @@
       <c r="E18" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="4" t="s">
         <v>130</v>
       </c>
     </row>
@@ -1221,7 +1236,7 @@
       <c r="E19" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" s="4" t="s">
         <v>131</v>
       </c>
     </row>
@@ -1241,7 +1256,7 @@
       <c r="E20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F20" s="6"/>
+      <c r="F20" s="4"/>
     </row>
     <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -1259,11 +1274,11 @@
       <c r="E21" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" s="4" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>57</v>
       </c>
@@ -1274,14 +1289,16 @@
         <v>59</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F22" s="6"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>60</v>
       </c>
@@ -1292,14 +1309,16 @@
         <v>59</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F23" s="6"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>62</v>
       </c>
@@ -1310,14 +1329,16 @@
         <v>59</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F24" s="6"/>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F24" s="4" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>64</v>
       </c>
@@ -1331,9 +1352,11 @@
         <v>10</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F25" s="6"/>
+        <v>137</v>
+      </c>
+      <c r="F25" s="4" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="26" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -1351,7 +1374,7 @@
       <c r="E26" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="4" t="s">
         <v>133</v>
       </c>
     </row>
@@ -1371,7 +1394,7 @@
       <c r="E27" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" s="4" t="s">
         <v>134</v>
       </c>
     </row>
@@ -1391,7 +1414,7 @@
       <c r="E28" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" s="4" t="s">
         <v>135</v>
       </c>
     </row>
@@ -1411,7 +1434,7 @@
       <c r="E29" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="4" t="s">
         <v>136</v>
       </c>
     </row>
@@ -1431,7 +1454,7 @@
       <c r="E30" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F30" s="6"/>
+      <c r="F30" s="4"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
@@ -1449,7 +1472,7 @@
       <c r="E31" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F31" s="6"/>
+      <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
@@ -1467,7 +1490,7 @@
       <c r="E32" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F32" s="6"/>
+      <c r="F32" s="4"/>
     </row>
     <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
@@ -1485,7 +1508,7 @@
       <c r="E33" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="F33" s="5" t="s">
         <v>112</v>
       </c>
     </row>
@@ -1505,7 +1528,7 @@
       <c r="E34" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="F34" s="4" t="s">
         <v>113</v>
       </c>
     </row>
@@ -1525,7 +1548,7 @@
       <c r="E35" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F35" s="4" t="s">
         <v>114</v>
       </c>
     </row>
@@ -1545,7 +1568,7 @@
       <c r="E36" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F36" s="6"/>
+      <c r="F36" s="4"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
@@ -1563,7 +1586,7 @@
       <c r="E37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F37" s="6"/>
+      <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
@@ -1581,7 +1604,7 @@
       <c r="E38" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F38" s="6"/>
+      <c r="F38" s="4"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
@@ -1599,7 +1622,7 @@
       <c r="E39" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F39" s="6"/>
+      <c r="F39" s="4"/>
     </row>
     <row r="40" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -1617,7 +1640,7 @@
       <c r="E40" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F40" s="6" t="s">
+      <c r="F40" s="4" t="s">
         <v>115</v>
       </c>
     </row>
@@ -1637,7 +1660,7 @@
       <c r="E41" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F41" s="6" t="s">
+      <c r="F41" s="4" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1657,7 +1680,7 @@
       <c r="E42" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F42" s="6" t="s">
+      <c r="F42" s="4" t="s">
         <v>117</v>
       </c>
     </row>
@@ -1677,7 +1700,7 @@
       <c r="E43" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="F43" s="6" t="s">
+      <c r="F43" s="4" t="s">
         <v>118</v>
       </c>
     </row>
@@ -1697,7 +1720,7 @@
       <c r="E44" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F44" s="6"/>
+      <c r="F44" s="4"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
@@ -1715,7 +1738,7 @@
       <c r="E45" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="F45" s="6"/>
+      <c r="F45" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat: Barcode, Reports, Receipt. feat: New Barcode Scanning feature. Allows the user to add an item to the cart via the barcode on the bottom of the catalogue panel. feat: Reports screen can now be used to get previous shift reports and allow the users to print them. feat: Receipts screen can now pull data from the server and be printed. (WIP: Needs to double check why receipts can not be previewed) feat: Users can now pick the Services from the Catalogue Panel. feat: Users can now pick the Packages from the Catalogue Panel. feat: Users can now pick the Addon from the Catalogue Panel. feat: Product Grid now shows the Services, Packages, and Addons pulled from the server.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70CC08D1-D961-4D79-B55C-DE3D0097FE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDF2F0D-90D1-44E7-BE3D-BB1ED6563D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="150">
   <si>
     <t>API Integration &amp; Testing Checklist</t>
   </si>
@@ -446,6 +446,30 @@
   </si>
   <si>
     <t>Used to refund the orders. The user is required to manually input the OR number as well as the reason for the refund.</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Unused by the original Application. (This is the same as discount/getactive API so this is redundancy.)</t>
+  </si>
+  <si>
+    <t>Unused by the original Application. (Passes detailid and discountid.)</t>
+  </si>
+  <si>
+    <t>Decided to not use since this API is most likely used for barcode scanner. I made use of the previous API to manually fetch it from local DB for the function to work without internet.</t>
+  </si>
+  <si>
+    <t>Used to fetch the reports data per shift from the server to localDB.</t>
+  </si>
+  <si>
+    <t>Used to fetch the receipts data from the server by datefrom and dateto.</t>
+  </si>
+  <si>
+    <t>WIP: PRINTING TEST SINCE PREVIEW DOESN'T WORK.</t>
+  </si>
+  <si>
+    <t>WIP: PRINTING NOT YET TESTED.</t>
   </si>
 </sst>
 </file>
@@ -491,7 +515,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -514,11 +538,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -535,6 +570,12 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -886,7 +927,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="39" customWidth="1"/>
@@ -894,6 +935,7 @@
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="30" customWidth="1"/>
+    <col min="7" max="7" width="28.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
@@ -986,7 +1028,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
@@ -1000,9 +1042,11 @@
         <v>18</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="4"/>
+        <v>142</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -1182,7 +1226,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>44</v>
       </c>
@@ -1196,11 +1240,13 @@
         <v>18</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" s="4"/>
-    </row>
-    <row r="18" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>46</v>
       </c>
@@ -1220,7 +1266,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
         <v>49</v>
       </c>
@@ -1240,7 +1286,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
         <v>52</v>
       </c>
@@ -1254,11 +1300,13 @@
         <v>10</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F20" s="4"/>
-    </row>
-    <row r="21" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>54</v>
       </c>
@@ -1278,7 +1326,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>57</v>
       </c>
@@ -1292,13 +1340,13 @@
         <v>10</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F22" s="4" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>60</v>
       </c>
@@ -1312,13 +1360,13 @@
         <v>10</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="105" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>62</v>
       </c>
@@ -1332,13 +1380,13 @@
         <v>10</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F24" s="4" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>64</v>
       </c>
@@ -1352,13 +1400,13 @@
         <v>10</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F25" s="4" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>66</v>
       </c>
@@ -1378,7 +1426,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>69</v>
       </c>
@@ -1398,7 +1446,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>71</v>
       </c>
@@ -1418,7 +1466,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>73</v>
       </c>
@@ -1438,7 +1486,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>75</v>
       </c>
@@ -1449,14 +1497,20 @@
         <v>14</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F30" s="4"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F30" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="H30" s="9"/>
+    </row>
+    <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>77</v>
       </c>
@@ -1467,14 +1521,20 @@
         <v>68</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" s="4"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="G31" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="H31" s="9"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>79</v>
       </c>
@@ -1744,7 +1804,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E45">
+  <conditionalFormatting sqref="E4:E45 G30:G31">
     <cfRule type="cellIs" dxfId="3" priority="1" stopIfTrue="1" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: New Cash Drop. feat: Added new cash drop dao, dto, dao provider, repository, and table for local DB management. feat: Added cash drop service to be able to be globally callable in case cash drop is to be used on different areas of the app. feat: Added cash drop controller to separate the functions from the dashboard controller. feat: Added cash drop generator for the user to print a cash drop report.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FDF2F0D-90D1-44E7-BE3D-BB1ED6563D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF20F204-D626-4BCF-A234-DC677D886AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="151">
   <si>
     <t>API Integration &amp; Testing Checklist</t>
   </si>
@@ -470,6 +470,9 @@
   </si>
   <si>
     <t>WIP: PRINTING NOT YET TESTED.</t>
+  </si>
+  <si>
+    <t>Unused?</t>
   </si>
 </sst>
 </file>
@@ -568,14 +571,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -939,14 +942,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1505,10 +1508,10 @@
       <c r="F30" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="G30" s="8" t="s">
+      <c r="G30" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="H30" s="9"/>
+      <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
@@ -1529,10 +1532,10 @@
       <c r="F31" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="G31" s="8" t="s">
+      <c r="G31" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="H31" s="9"/>
+      <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
@@ -1626,9 +1629,11 @@
         <v>10</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F36" s="4"/>
+        <v>137</v>
+      </c>
+      <c r="F36" s="4" t="s">
+        <v>150</v>
+      </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">

</xml_diff>

<commit_message>
feat: Send Cash Report. feat: Send cash report dao, dto, dao provider, repository, table. feat: Send cash report will be sent during end shift after the cash drop call and end shift API call. feat: updated service to support cash report call. feat: updated dashboard controller to call the service during end shift.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF20F204-D626-4BCF-A234-DC677D886AC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108D7AE9-C308-4F5D-8282-01CBC3AAC970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="154">
   <si>
     <t>API Integration &amp; Testing Checklist</t>
   </si>
@@ -473,6 +473,15 @@
   </si>
   <si>
     <t>Unused?</t>
+  </si>
+  <si>
+    <t>Potentially Unused.</t>
+  </si>
+  <si>
+    <t>Used to send Ending Cash report from application to the server. This is sent AFTER the end shift and cash drop.</t>
+  </si>
+  <si>
+    <t>Used to get cash reports from the server to the application's cash report screen.</t>
   </si>
 </sst>
 </file>
@@ -1649,11 +1658,13 @@
         <v>89</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F37" s="4"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+      <c r="F37" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>94</v>
       </c>
@@ -1664,14 +1675,16 @@
         <v>86</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F38" s="4"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+      <c r="F38" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
         <v>96</v>
       </c>
@@ -1682,12 +1695,14 @@
         <v>86</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F39" s="4"/>
+        <v>137</v>
+      </c>
+      <c r="F39" s="4" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="40" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
@@ -1700,7 +1715,7 @@
         <v>100</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E40" s="3" t="s">
         <v>111</v>
@@ -1720,7 +1735,7 @@
         <v>100</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E41" s="3" t="s">
         <v>111</v>
@@ -1740,7 +1755,7 @@
         <v>100</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E42" s="3" t="s">
         <v>111</v>
@@ -1760,7 +1775,7 @@
         <v>100</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E43" s="3" t="s">
         <v>111</v>
@@ -1780,7 +1795,7 @@
         <v>100</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>89</v>
+        <v>10</v>
       </c>
       <c r="E44" s="3" t="s">
         <v>11</v>

</xml_diff>

<commit_message>
feat: Customer and Cash Report. feat: Added Cash Reporting for the user to be able to view cash reports per shift on a specific business date. feat: Added Indivual/Company creation on the application. feat: Added Customer Creation UI on the POS.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108D7AE9-C308-4F5D-8282-01CBC3AAC970}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CF2420-6B80-42F9-9C8F-912D8372FFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="API Checklist" sheetId="1" r:id="rId1"/>
@@ -466,12 +466,6 @@
     <t>Used to fetch the receipts data from the server by datefrom and dateto.</t>
   </si>
   <si>
-    <t>WIP: PRINTING TEST SINCE PREVIEW DOESN'T WORK.</t>
-  </si>
-  <si>
-    <t>WIP: PRINTING NOT YET TESTED.</t>
-  </si>
-  <si>
     <t>Unused?</t>
   </si>
   <si>
@@ -482,6 +476,12 @@
   </si>
   <si>
     <t>Used to get cash reports from the server to the application's cash report screen.</t>
+  </si>
+  <si>
+    <t>Used for Reprinting. Already using the getDetailID API for this. Redundant.</t>
+  </si>
+  <si>
+    <t>Used to send Customer Individual information and Company Information to track sales.</t>
   </si>
 </sst>
 </file>
@@ -1080,7 +1080,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>23</v>
       </c>
@@ -1094,9 +1094,11 @@
         <v>18</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="4"/>
+        <v>142</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>152</v>
+      </c>
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -1512,14 +1514,12 @@
         <v>10</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F30" s="4" t="s">
         <v>147</v>
       </c>
-      <c r="G30" s="6" t="s">
-        <v>148</v>
-      </c>
+      <c r="G30" s="6"/>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
@@ -1536,14 +1536,12 @@
         <v>10</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="G31" s="6" t="s">
-        <v>149</v>
-      </c>
+      <c r="G31" s="6"/>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
@@ -1641,7 +1639,7 @@
         <v>137</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -1661,7 +1659,7 @@
         <v>137</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="60" x14ac:dyDescent="0.25">
@@ -1681,7 +1679,7 @@
         <v>111</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="45" x14ac:dyDescent="0.25">
@@ -1698,10 +1696,10 @@
         <v>10</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>137</v>
+        <v>111</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="30" x14ac:dyDescent="0.25">
@@ -1784,7 +1782,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
         <v>107</v>
       </c>
@@ -1798,9 +1796,11 @@
         <v>10</v>
       </c>
       <c r="E44" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F44" s="4"/>
+        <v>111</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>153</v>
+      </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">

</xml_diff>

<commit_message>
feat: New Split Payment E2E complete. feat: Loading state for payment to avoid duplications. feat: Idempotency on every transaction so no duplications can ever happen. feat: garbage collection on sales and split payments table for data longer than 7 days.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CF2420-6B80-42F9-9C8F-912D8372FFC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{695E1269-6DCC-4DCB-AEFB-15B68E1AD356}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="155">
   <si>
     <t>API Integration &amp; Testing Checklist</t>
   </si>
@@ -482,6 +482,9 @@
   </si>
   <si>
     <t>Used to send Customer Individual information and Company Information to track sales.</t>
+  </si>
+  <si>
+    <t>Used separate from Sales. This will handle E2E payments from application to server.</t>
   </si>
 </sst>
 </file>
@@ -1544,7 +1547,7 @@
       <c r="G31" s="6"/>
       <c r="H31" s="7"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
         <v>79</v>
       </c>
@@ -1558,9 +1561,11 @@
         <v>10</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F32" s="4"/>
+        <v>137</v>
+      </c>
+      <c r="F32" s="4" t="s">
+        <v>154</v>
+      </c>
     </row>
     <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">

</xml_diff>

<commit_message>
fix: Locks dashboard if there's no Shift. fix: Updated shift on top bar to show users that the shift is inactive.
</commit_message>
<xml_diff>
--- a/gpos_provantis/API_Checklist.xlsx
+++ b/gpos_provantis/API_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS\gpos-provantis\gpos_provantis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E87628C1-34E3-49E5-9A2E-A1B142CE365F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{092413CA-F0A7-4E89-BD4A-23702FC02536}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="API Checklist" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="154">
   <si>
     <t>API Integration &amp; Testing Checklist</t>
   </si>
@@ -55,9 +55,6 @@
     <t>POST</t>
   </si>
   <si>
-    <t>Pending</t>
-  </si>
-  <si>
     <t>salesDetailAPI</t>
   </si>
   <si>
@@ -433,9 +430,6 @@
     <t>Used to show the amount collected by the cashier inside the receipt.</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>Used to get services for the application to be able to use.</t>
   </si>
   <si>
@@ -448,9 +442,6 @@
     <t>Used to refund the orders. The user is required to manually input the OR number as well as the reason for the refund.</t>
   </si>
   <si>
-    <t>Failed</t>
-  </si>
-  <si>
     <t>Unused by the original Application. (This is the same as discount/getactive API so this is redundancy.)</t>
   </si>
   <si>
@@ -478,13 +469,19 @@
     <t>Used to get cash reports from the server to the application's cash report screen.</t>
   </si>
   <si>
-    <t>Used for Reprinting. Already using the getDetailID API for this. Redundant.</t>
-  </si>
-  <si>
     <t>Used to send Customer Individual information and Company Information to track sales.</t>
   </si>
   <si>
     <t>Used separate from Sales. This will handle E2E payments from application to server.</t>
+  </si>
+  <si>
+    <t>Used to bind customer purchase order to an order.</t>
+  </si>
+  <si>
+    <t>Used for reprinting by sending the OR number to the API.</t>
+  </si>
+  <si>
+    <t>Skipped</t>
   </si>
 </sst>
 </file>
@@ -997,107 +994,107 @@
         <v>10</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>14</v>
-      </c>
       <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E6" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="C7" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="E7" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>142</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>24</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>142</v>
+        <v>110</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>152</v>
@@ -1105,731 +1102,733 @@
     </row>
     <row r="10" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="D10" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="D11" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="D12" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="D13" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>38</v>
-      </c>
       <c r="C14" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="C15" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>43</v>
-      </c>
       <c r="D16" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>45</v>
-      </c>
       <c r="C17" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="C18" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>48</v>
-      </c>
       <c r="D18" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B19" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="C19" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>51</v>
-      </c>
       <c r="D19" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>53</v>
-      </c>
       <c r="C20" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D20" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="D21" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>59</v>
-      </c>
       <c r="D22" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="C23" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="105" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>63</v>
-      </c>
       <c r="C24" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>65</v>
-      </c>
       <c r="C25" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C26" s="3" t="s">
-        <v>68</v>
-      </c>
       <c r="D26" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>70</v>
-      </c>
       <c r="C27" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>72</v>
-      </c>
       <c r="C28" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>74</v>
-      </c>
       <c r="C29" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="30" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>76</v>
-      </c>
       <c r="C30" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="G30" s="6"/>
       <c r="H30" s="7"/>
     </row>
     <row r="31" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B31" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="C31" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="7"/>
     </row>
     <row r="32" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>80</v>
-      </c>
       <c r="C32" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>137</v>
+        <v>110</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B33" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B33" s="2" t="s">
+      <c r="C33" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C33" s="3" t="s">
-        <v>83</v>
-      </c>
       <c r="D33" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E33" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33" s="5" t="s">
         <v>111</v>
-      </c>
-      <c r="F33" s="5" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B34" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="C34" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C34" s="3" t="s">
-        <v>86</v>
-      </c>
       <c r="D34" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="35" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B35" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="2" t="s">
+      <c r="C35" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C35" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="3" t="s">
-        <v>89</v>
-      </c>
       <c r="E35" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B36" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>91</v>
-      </c>
       <c r="C36" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B37" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>93</v>
-      </c>
       <c r="C37" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E37" s="3" t="s">
-        <v>137</v>
+        <v>153</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>95</v>
-      </c>
       <c r="C38" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E38" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="C39" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B40" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="C40" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="C40" s="3" t="s">
-        <v>100</v>
-      </c>
       <c r="D40" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E40" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B41" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>102</v>
-      </c>
       <c r="C41" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E41" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B42" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="C42" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E42" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="C43" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E43" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B44" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B44" s="2" t="s">
+      <c r="C44" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E44" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="C44" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="D44" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="E44" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
+      <c r="B45" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="C45" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>10</v>
       </c>
       <c r="E45" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="F45" s="4"/>
+        <v>110</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>151</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:E45 G30:G31">
+  <conditionalFormatting sqref="G30:G31 E4:E45">
     <cfRule type="cellIs" dxfId="3" priority="1" stopIfTrue="1" operator="equal">
       <formula>"Passed"</formula>
     </cfRule>

</xml_diff>